<commit_message>
docs: WBS GitHub 등록 자산 추가(담당자 배정 + Issues/Milestones/Projects)
- docs/08-wbs.md, 08-wbs.xlsx: 담당자 열 추가(PM·PL·개발자 A~E, 381개 작업)
- docs/09-wbs-github.md: 등록 가이드(담당자 정책·마일스톤 20·라벨·이슈 55 목록)
- docs/wbs-github-issues.csv: 작업패키지 55개 임포트용 CSV
- scripts/import-wbs-github.sh: gh CLI 자동 등록 스크립트(라벨/마일스톤/이슈/프로젝트)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/08-wbs.xlsx
+++ b/docs/08-wbs.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt_Chart" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$4:$I$385</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WBS'!$A$4:$J$385</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,8 +65,13 @@
       <name val="맑은 고딕"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="25">
+  <fills count="32">
     <fill>
       <patternFill/>
     </fill>
@@ -188,6 +193,41 @@
         <fgColor rgb="0044557A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000052CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001D76DB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000E8A16"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B60205"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D93F0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006F42C1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005319E7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -259,7 +299,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -355,6 +395,27 @@
     <xf numFmtId="0" fontId="0" fillId="23" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -841,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I386"/>
+  <dimension ref="A1:J386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -853,6 +914,7 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -915,6 +977,11 @@
           <t>세부사항</t>
         </is>
       </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>담당자</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -958,6 +1025,11 @@
           <t>모노레포 Git 저장소 초기화. .gitignore(node_modules·.env·빌드 산출물·.expo), README에 서비스 개요·로컬 실행법·환경 구성 명시. 참고: CLAUDE.md(하네스 정의)</t>
         </is>
       </c>
+      <c r="J5" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -1001,6 +1073,11 @@
           <t>프론트(Next.js App Router)·모바일(Expo RN)·백엔드(Supabase/bkend.ai)·DB(PostgreSQL+RLS) 스택 확정 및 근거 문서화. 참고: docs/02-data-specification.md, docs/03-erd.md</t>
         </is>
       </c>
+      <c r="J6" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -1044,6 +1121,11 @@
           <t>apps/web 에 Next.js App Router 프로젝트 부팅(라우팅·서버컴포넌트 구조). 참고: docs/06-information-architecture.md §4 반응형 웹 IA</t>
         </is>
       </c>
+      <c r="J7" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -1087,6 +1169,11 @@
           <t>apps/mobile 에 Expo 기반 RN 앱 부팅(네비게이션 스택·탭). 참고: docs/06-information-architecture.md §5 모바일 앱 IA</t>
         </is>
       </c>
+      <c r="J8" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -1130,6 +1217,11 @@
           <t>Supabase 프로젝트 생성 후 dev/stg/prod 3환경 분리(.env.dev/.stg/.prod). 키·URL 환경변수화. 참고: docs/03-erd.md §RLS 정책 요약</t>
         </is>
       </c>
+      <c r="J9" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -1173,6 +1265,11 @@
           <t>bkend.ai BaaS(또는 Supabase 직접) 클라이언트 래퍼 구현 — 인증·DB·스토리지 SDK 초기화. 참고: docs/02-data-specification.md §1 테이블 목록, bkit:bkend-quickstart 스킬</t>
         </is>
       </c>
+      <c r="J10" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -1216,6 +1313,11 @@
           <t>TypeScript strict + ESLint + Prettier 규칙 정립(AI 협업용 코딩 컨벤션). 참고: bkit:phase-2-convention 스킬</t>
         </is>
       </c>
+      <c r="J11" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -1259,6 +1361,11 @@
           <t>도메인 기반 폴더 구조(features/·lib/·components/·app/) 컨벤션 문서화.</t>
         </is>
       </c>
+      <c r="J12" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -1302,6 +1409,11 @@
           <t>pnpm workspaces 로 web·mobile·shared(타입·API 클라이언트·검증 스키마) 패키지 공유 구성.</t>
         </is>
       </c>
+      <c r="J13" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -1345,6 +1457,11 @@
           <t>Vercel(웹)·EAS/Render(모바일·서버) 배포 환경 사전 셋업. 참고: docs/08-wbs.md §19 CI/CD</t>
         </is>
       </c>
+      <c r="J14" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1388,6 +1505,11 @@
           <t>Sentry 연동 — 웹·모바일·서버 런타임 에러 트래킹 및 소스맵 업로드.</t>
         </is>
       </c>
+      <c r="J15" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -1431,6 +1553,11 @@
           <t>i18n 셋업(한국어 기본, 영어 차기 릴리스). 참고: docs/07-design-system.md §2 타이포그래피(Pretendard)</t>
         </is>
       </c>
+      <c r="J16" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n">
@@ -1474,6 +1601,11 @@
           <t>users 테이블 — 모든 역할(보호자·당사자·전문가)의 계정. role enum·email·phone·status. 참고: docs/02-data-specification.md §2 핵심 테이블 상세(users), docs/03-erd.md</t>
         </is>
       </c>
+      <c r="J17" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
@@ -1517,6 +1649,11 @@
           <t>persons 테이블 — 기록의 주체인 당사자. birth_date·life_stage(생애주기)·emergency_info(JSONB). 참고: docs/02 §2(persons), §4 Enum(life_stage)</t>
         </is>
       </c>
+      <c r="J18" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n">
@@ -1560,6 +1697,11 @@
           <t>guardian_persons — 보호자↔당사자 N:M 매핑, is_primary(주보호자)·relationship. 참고: docs/02 §2(guardian_persons), docs/03-erd.md §도메인별 서브 ERD</t>
         </is>
       </c>
+      <c r="J19" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n">
@@ -1603,6 +1745,11 @@
           <t>person_accounts — 당사자 선택적 로그인 계정 + 접근성 설정(ui_mode·font_scale·contrast). 참고: docs/02 §2(person_accounts), docs/07 §9 당사자 접근성 모드</t>
         </is>
       </c>
+      <c r="J20" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n">
@@ -1646,6 +1793,11 @@
           <t>permissions — 권한 매트릭스 핵심. domain·access_level·valid_from/until. 참고: docs/02 §2(permissions), §4 Enum(domain·access_level)</t>
         </is>
       </c>
+      <c r="J21" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
@@ -1689,6 +1841,11 @@
           <t>permission_logs — 권한 부여/수정/회수 이력(감사 추적). 참고: docs/02 §2(permission_logs), docs/05-workflows-feature.md §2·§3</t>
         </is>
       </c>
+      <c r="J22" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n">
@@ -1732,6 +1889,11 @@
           <t>records — 6도메인 기록 공통 테이블. domain·record_type·content(JSONB)·is_draft·is_milestone. 참고: docs/02 §2(records), §3 JSONB content 스키마</t>
         </is>
       </c>
+      <c r="J23" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
@@ -1775,6 +1937,11 @@
           <t>self_expressions — 당사자 자기표현(날짜별 UNIQUE). mood·activities·content(JSONB). 참고: docs/02 §2(self_expressions), §3 JSONB</t>
         </is>
       </c>
+      <c r="J24" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n">
@@ -1818,6 +1985,11 @@
           <t>record_files — 기록·자기표현 첨부 파일 메타. storage_path·sensitivity·mime. 참고: docs/02 §2(record_files), docs/05 §5 파일 첨부</t>
         </is>
       </c>
+      <c r="J25" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
@@ -1861,6 +2033,11 @@
           <t>life_milestones — 생애주기 이정표(진단·입학·졸업 등). category·event_date. 참고: docs/02 §2(life_milestones), docs/05 §6 타임라인</t>
         </is>
       </c>
+      <c r="J26" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n">
@@ -1904,6 +2081,11 @@
           <t>handovers — 전문가 인수인계. domain·summary·linked_record_ids·is_confirmed. 참고: docs/02 §2(handovers), docs/05 §7 인수인계</t>
         </is>
       </c>
+      <c r="J27" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
@@ -1947,6 +2129,11 @@
           <t>access_logs — INSERT-only 접근 로그(불변). actor·action·target. 참고: docs/02 §2(access_logs), docs/03 §RLS 정책 요약</t>
         </is>
       </c>
+      <c r="J28" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n">
@@ -1990,6 +2177,11 @@
           <t>notifications — 알림. type·payload(JSONB)·self_expression_id FK·is_read. 참고: docs/02 §2(notifications), §3 JSONB, docs/05 §8 알림</t>
         </is>
       </c>
+      <c r="J29" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
@@ -2033,6 +2225,11 @@
           <t>records SELECT RLS — 보호자(매핑)·당사자 본인·권한자(permissions 유효기간 내)만 조회. 참고: docs/03 §RLS 정책 요약, docs/02 §6 제약조건</t>
         </is>
       </c>
+      <c r="J30" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n">
@@ -2076,6 +2273,11 @@
           <t>records INSERT/UPDATE RLS — 도메인·access_level(write 이상) 검증. 참고: docs/03 §RLS, docs/05 §4 기록 작성 공통</t>
         </is>
       </c>
+      <c r="J31" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
@@ -2119,6 +2321,11 @@
           <t>self_expressions RLS — 당사자 본인 계정만 작성/수정(당일). 참고: docs/03 §RLS, docs/04-workflows-user.md §2 당사자</t>
         </is>
       </c>
+      <c r="J32" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n">
@@ -2162,6 +2369,11 @@
           <t>access_logs INSERT-only 정책 — UPDATE/DELETE 차단으로 로그 불변성 보장. 참고: docs/03 §RLS, docs/08-wbs.md §17.2.8</t>
         </is>
       </c>
+      <c r="J33" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n">
@@ -2203,6 +2415,11 @@
       <c r="I34" s="33" t="inlineStr">
         <is>
           <t>permissions 변경 RLS — 주보호자만 권한 부여/회수 가능. 참고: docs/03 §RLS, docs/05 §2 권한 부여</t>
+        </is>
+      </c>
+      <c r="J34" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
         </is>
       </c>
     </row>
@@ -2248,6 +2465,11 @@
           <t>이메일/비밀번호 회원가입. role 선택 분기(보호자·당사자·전문가). users insert + 이메일 인증 트리거. 참고: docs/05 §1 회원가입 &amp; 역할별 온보딩, wireframes/web/11-signup-role.svg·12-signup-profile.svg</t>
         </is>
       </c>
+      <c r="J35" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
@@ -2291,6 +2513,11 @@
           <t>이메일/비밀번호 로그인 + JWT 발급·세션. 참고: docs/04 §7 역할별 진입점 비교, wireframes/web/01-login.svg, bkit:bkend-auth 스킬</t>
         </is>
       </c>
+      <c r="J36" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -2334,6 +2561,11 @@
           <t>로그아웃 — 세션/토큰 무효화. 참고: bkit:bkend-auth 스킬</t>
         </is>
       </c>
+      <c r="J37" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
@@ -2377,6 +2609,11 @@
           <t>이메일 인증 메일 발송(토큰 생성·만료). 참고: docs/05 §1, wireframes/web/13-signup-verify.svg</t>
         </is>
       </c>
+      <c r="J38" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="n">
@@ -2420,6 +2657,11 @@
           <t>이메일 인증 토큰 확인 + users.status 활성화. 참고: docs/05 §1 온보딩, wireframes/web/13-signup-verify.svg</t>
         </is>
       </c>
+      <c r="J39" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n">
@@ -2463,6 +2705,11 @@
           <t>비밀번호 재설정 요청(재설정 토큰 메일). 참고: wireframes/web/15-reset-password.svg</t>
         </is>
       </c>
+      <c r="J40" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n">
@@ -2506,6 +2753,11 @@
           <t>비밀번호 재설정 확인 + 해시 갱신. 참고: wireframes/web/15-reset-password.svg</t>
         </is>
       </c>
+      <c r="J41" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n">
@@ -2549,6 +2801,11 @@
           <t>초대 링크 생성 — 보호자가 전문가/공동보호자 초대(토큰·도메인·만료). 참고: docs/05 §1 온보딩·§2 권한 부여</t>
         </is>
       </c>
+      <c r="J42" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="n">
@@ -2592,6 +2849,11 @@
           <t>초대 링크 수락 — 토큰 검증 후 신규 가입 또는 기존 계정 연결 분기 + 권한 자동 매핑. 참고: docs/05 §1, wireframes/web/14-invite-accept.svg</t>
         </is>
       </c>
+      <c r="J43" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n">
@@ -2635,6 +2897,11 @@
           <t>카카오 OAuth 소셜 로그인(P1). 참고: docs/04 §7 진입점, bkit:bkend-auth 스킬</t>
         </is>
       </c>
+      <c r="J44" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n">
@@ -2678,6 +2945,11 @@
           <t>네이버 OAuth 소셜 로그인(P1). 참고: docs/04 §7 진입점, bkit:bkend-auth 스킬</t>
         </is>
       </c>
+      <c r="J45" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="n">
@@ -2721,6 +2993,11 @@
           <t>사용자 본인/타 사용자 프로필 단건 조회(권한 범위 내). 참고: docs/02 §2(users)</t>
         </is>
       </c>
+      <c r="J46" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="12" t="n">
@@ -2764,6 +3041,11 @@
           <t>사용자 프로필 수정(이름·연락처·프로필 사진). 참고: wireframes/web/24-guardian-profile-edit.svg</t>
         </is>
       </c>
+      <c r="J47" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="n">
@@ -2807,6 +3089,11 @@
           <t>사용자 soft delete(status=inactive) — 데이터 보존, 로그인 차단. 참고: docs/02 §4 Enum(user status)</t>
         </is>
       </c>
+      <c r="J48" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="n">
@@ -2850,6 +3137,11 @@
           <t>이메일·전화번호로 사용자 검색(초대·권한 부여 시). 참고: docs/05 §2 권한 부여 Step1</t>
         </is>
       </c>
+      <c r="J49" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="n">
@@ -2893,6 +3185,11 @@
           <t>역할 기반 사용자 필터(전문가 유형별 등, P1).</t>
         </is>
       </c>
+      <c r="J50" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="12" t="n">
@@ -2936,6 +3233,11 @@
           <t>당사자 신규 등록 — 기본정보·생애주기·응급정보 입력 + guardian_persons 자동 연결. 참고: docs/02 §2(persons), docs/04 §1 보호자, wireframes/web/17-guardian-person-register.svg</t>
         </is>
       </c>
+      <c r="J51" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="n">
@@ -2979,6 +3281,11 @@
           <t>당사자 상세 조회(프로필·요약). 참고: wireframes/web/16-guardian-person-profile.svg</t>
         </is>
       </c>
+      <c r="J52" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="n">
@@ -3022,6 +3329,11 @@
           <t>보호자 기준 담당 당사자 목록(대시보드 진입점). 참고: docs/04 §1 보호자, wireframes/web/02-guardian-dashboard.svg</t>
         </is>
       </c>
+      <c r="J53" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="n">
@@ -3065,6 +3377,11 @@
           <t>당사자 기본정보 수정. 참고: wireframes/web/25-guardian-person-edit.svg</t>
         </is>
       </c>
+      <c r="J54" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="12" t="n">
@@ -3108,6 +3425,11 @@
           <t>당사자 응급정보(혈액형·알레르기·복약·비상연락) 수정 — 추가 인증 필요. 참고: docs/02 §3 JSONB(emergency), docs/08-wbs.md §17.2.5, wireframes/web/26-guardian-emergency-edit.svg</t>
         </is>
       </c>
+      <c r="J55" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="12" t="n">
@@ -3151,6 +3473,11 @@
           <t>당사자 프로필 사진 업로드(presigned URL). 참고: docs/05 §5 파일 첨부</t>
         </is>
       </c>
+      <c r="J56" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="12" t="n">
@@ -3194,6 +3521,11 @@
           <t>당사자 프로필 사진 삭제(storage+meta).</t>
         </is>
       </c>
+      <c r="J57" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="12" t="n">
@@ -3237,6 +3569,11 @@
           <t>당사자 비활성화/이장(archive) — 사망·이전 등(P1). 참고: docs/05 §10 당사자 전환기 처리</t>
         </is>
       </c>
+      <c r="J58" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="n">
@@ -3280,6 +3617,11 @@
           <t>birth_date 기반 life_stage 자동 계산 DB 트리거(영유아~노년 6단계). 참고: docs/01-record-matrix.md, docs/02 §4 Enum(life_stage)</t>
         </is>
       </c>
+      <c r="J59" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="12" t="n">
@@ -3323,6 +3665,11 @@
           <t>보호자-당사자 연결 생성(관계·주보호자 여부). 참고: docs/02 §2(guardian_persons)</t>
         </is>
       </c>
+      <c r="J60" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="n">
@@ -3366,6 +3713,11 @@
           <t>보호자-당사자 매핑 단건 조회.</t>
         </is>
       </c>
+      <c r="J61" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="12" t="n">
@@ -3409,6 +3761,11 @@
           <t>당사자별 보호자 목록(공동 양육 지원). 참고: docs/03 §도메인별 서브 ERD</t>
         </is>
       </c>
+      <c r="J62" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="12" t="n">
@@ -3452,6 +3809,11 @@
           <t>주보호자(is_primary) 변경 — 단일 주보호자 제약. 참고: docs/02 §6 제약조건</t>
         </is>
       </c>
+      <c r="J63" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="12" t="n">
@@ -3495,6 +3857,11 @@
           <t>관계(부/모/후견인 등) 수정. 참고: docs/02 §4 Enum(relationship)</t>
         </is>
       </c>
+      <c r="J64" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="12" t="n">
@@ -3538,6 +3905,11 @@
           <t>보호자 연결 해제(P1).</t>
         </is>
       </c>
+      <c r="J65" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="12" t="n">
@@ -3581,6 +3953,11 @@
           <t>당사자 선택적 로그인 계정 생성(자기표현·내 기록용). 참고: docs/02 §2(person_accounts), docs/04 §2 당사자</t>
         </is>
       </c>
+      <c r="J66" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="12" t="n">
@@ -3624,6 +4001,11 @@
           <t>당사자 접근성 설정 조회. 참고: wireframes/web/33-person-profile.svg</t>
         </is>
       </c>
+      <c r="J67" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="12" t="n">
@@ -3667,6 +4049,11 @@
           <t>접근성 설정 수정(글씨 크기·고대비·TTS). 참고: docs/07 §9 당사자 접근성 모드, wireframes/web/32-person-accessibility.svg</t>
         </is>
       </c>
+      <c r="J68" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="12" t="n">
@@ -3710,6 +4097,11 @@
           <t>UI 모드(아이콘 전용/혼합) 전환. 참고: docs/07 §9, docs/06 §1 스크린 유형</t>
         </is>
       </c>
+      <c r="J69" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="13" t="n">
@@ -3753,6 +4145,11 @@
           <t>권한 부여 — 권한자·도메인(멀티)·수준(read/write/manage)·기간 UPSERT. 참고: docs/02 §2(permissions)·§4 Enum, docs/05 §2 권한 부여</t>
         </is>
       </c>
+      <c r="J70" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="13" t="n">
@@ -3796,6 +4193,11 @@
           <t>권한 단건 조회.</t>
         </is>
       </c>
+      <c r="J71" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="13" t="n">
@@ -3839,6 +4241,11 @@
           <t>당사자별 권한 매트릭스(이해관계자×도메인 그리드). 참고: docs/05 §2, wireframes/web/07-permission-matrix.svg</t>
         </is>
       </c>
+      <c r="J72" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="13" t="n">
@@ -3882,6 +4289,11 @@
           <t>사용자(전문가)별 받은 권한 목록. 참고: wireframes/web/20-guardian-stakeholder-detail.svg</t>
         </is>
       </c>
+      <c r="J73" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="13" t="n">
@@ -3925,6 +4337,11 @@
           <t>권한 수정(수준·기간 변경) + permission_logs 기록. 참고: wireframes/web/28-guardian-permission-modals.svg</t>
         </is>
       </c>
+      <c r="J74" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="13" t="n">
@@ -3968,6 +4385,11 @@
           <t>권한 즉시 회수 + 캐시 무효화 + 알림. 참고: docs/05 §3 권한 회수 프로세스, wireframes/web/28-guardian-permission-modals.svg</t>
         </is>
       </c>
+      <c r="J75" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="13" t="n">
@@ -4011,6 +4433,11 @@
           <t>valid_until 만료 권한 자동 회수 cron(scheduled fn). 참고: docs/05 §3 권한 회수</t>
         </is>
       </c>
+      <c r="J76" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="13" t="n">
@@ -4054,6 +4481,11 @@
           <t>권한 만료 7일 전 사전 알림 cron(P1). 참고: docs/05 §8 알림</t>
         </is>
       </c>
+      <c r="J77" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="13" t="n">
@@ -4097,6 +4529,11 @@
           <t>권한 위자드 Step1 — 대상자 검색 또는 이메일 초대. 참고: docs/06 §6 주요 플로우(권한 부여), wireframes/web/21-guardian-grant-wizard.svg</t>
         </is>
       </c>
+      <c r="J78" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="13" t="n">
@@ -4140,6 +4577,11 @@
           <t>Step2 — 6개 도메인 멀티 선택. 참고: wireframes/web/21-guardian-grant-wizard.svg</t>
         </is>
       </c>
+      <c r="J79" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="13" t="n">
@@ -4183,6 +4625,11 @@
           <t>Step3 — 도메인별 접근 수준·유효 기간 설정. 참고: wireframes/web/21-guardian-grant-wizard.svg</t>
         </is>
       </c>
+      <c r="J80" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="13" t="n">
@@ -4226,6 +4673,11 @@
           <t>Step4 — 미리보기 후 permissions UPSERT + 알림 발송. 참고: docs/05 §2, wireframes/web/21-guardian-grant-wizard.svg</t>
         </is>
       </c>
+      <c r="J81" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="13" t="n">
@@ -4269,6 +4721,11 @@
           <t>permissions 변경 시 permission_logs 자동 기록 트리거. 참고: docs/02 §2(permission_logs)</t>
         </is>
       </c>
+      <c r="J82" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="13" t="n">
@@ -4312,6 +4769,11 @@
           <t>당사자별 권한 변경 이력 조회. 참고: docs/05 §9 접근 로그</t>
         </is>
       </c>
+      <c r="J83" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="13" t="n">
@@ -4355,6 +4817,11 @@
           <t>사용자별 권한 변동 이력 조회.</t>
         </is>
       </c>
+      <c r="J84" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="13" t="n">
@@ -4398,6 +4865,11 @@
           <t>권한 외 리소스 접근 시도 감지 트리거(RLS 위반 로깅). 참고: docs/03 §RLS, docs/05 §11 시스템 보안 흐름</t>
         </is>
       </c>
+      <c r="J85" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="13" t="n">
@@ -4441,6 +4913,11 @@
           <t>이상 접근 감지 시 보호자 알림 발송. 참고: docs/05 §8·§11</t>
         </is>
       </c>
+      <c r="J86" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="13" t="n">
@@ -4484,6 +4961,11 @@
           <t>권한 변경 시 Redis 권한 캐시 무효화(P1).</t>
         </is>
       </c>
+      <c r="J87" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="14" t="n">
@@ -4527,6 +5009,11 @@
           <t>도메인 무관 기록 생성 API — content(JSONB)는 record_type별 스키마 검증. 참고: docs/02 §3 JSONB content 스키마, docs/05 §4 기록 작성 공통, wireframes/web/06-record-form.svg</t>
         </is>
       </c>
+      <c r="J88" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="14" t="n">
@@ -4570,6 +5057,11 @@
           <t>기록 단건 조회(권한 검증). 참고: wireframes/web/05-record-detail.svg</t>
         </is>
       </c>
+      <c r="J89" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="14" t="n">
@@ -4613,6 +5105,11 @@
           <t>당사자별 전체 기록 목록(페이징·필터·정렬). 참고: docs/02 §5 인덱스 전략, wireframes/web/04-record-list.svg</t>
         </is>
       </c>
+      <c r="J90" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="14" t="n">
@@ -4656,6 +5153,11 @@
           <t>도메인별 기록 목록. 참고: wireframes/web/18-guardian-records-domain.svg</t>
         </is>
       </c>
+      <c r="J91" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="14" t="n">
@@ -4699,6 +5201,11 @@
           <t>기록 수정(작성자/권한자). 참고: wireframes/web/19-guardian-record-edit.svg</t>
         </is>
       </c>
+      <c r="J92" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="14" t="n">
@@ -4742,6 +5249,11 @@
           <t>기록 삭제(보호자 권한). 참고: docs/03 §RLS</t>
         </is>
       </c>
+      <c r="J93" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="14" t="n">
@@ -4785,6 +5297,11 @@
           <t>기록 임시저장(is_draft) — 위자드 중간 저장. 참고: docs/05 §4 기록 작성 공통</t>
         </is>
       </c>
+      <c r="J94" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="14" t="n">
@@ -4828,6 +5345,11 @@
           <t>기록을 이정표(is_milestone)로 표시 → 타임라인 강조. 참고: docs/05 §6 타임라인</t>
         </is>
       </c>
+      <c r="J95" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="n">
@@ -4871,6 +5393,11 @@
           <t>기록 고정/해제(상단 핀). 참고: docs/02 §2(records)</t>
         </is>
       </c>
+      <c r="J96" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="14" t="n">
@@ -4914,6 +5441,11 @@
           <t>기록 태그 추가/제거(P1).</t>
         </is>
       </c>
+      <c r="J97" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="n">
@@ -4957,6 +5489,11 @@
           <t>전문 검색(content 텍스트, P1). 참고: docs/02 §5 인덱스 전략(GIN)</t>
         </is>
       </c>
+      <c r="J98" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="14" t="n">
@@ -5000,6 +5537,11 @@
           <t>기록 일괄 PDF/CSV 내보내기(P1). 참고: docs/05 §6 타임라인 PDF</t>
         </is>
       </c>
+      <c r="J99" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="n">
@@ -5043,6 +5585,11 @@
           <t>작성자별 기록 통계 카운트(P2).</t>
         </is>
       </c>
+      <c r="J100" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="14" t="n">
@@ -5086,6 +5633,11 @@
           <t>MED-001 초기 진단 요약(보호자 작성). content JSONB: 진단명·진단일·기관. 참고: docs/01-record-matrix.md §1 영유아기, docs/02 §3 JSONB(MED-001)</t>
         </is>
       </c>
+      <c r="J101" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="n">
@@ -5129,6 +5681,11 @@
           <t>MED-002 발달 검사 결과(보호자). 검사도구·점수·해석. 참고: docs/01 §1·§2, docs/02 §3 JSONB(MED-002)</t>
         </is>
       </c>
+      <c r="J102" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="14" t="n">
@@ -5172,6 +5729,11 @@
           <t>MED-003 복약 기록(보호자). 약물·용량·주기·부작용. 참고: docs/02 §3 JSONB(MED-003)</t>
         </is>
       </c>
+      <c r="J103" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="n">
@@ -5215,6 +5777,11 @@
           <t>MED-004 응급 대응 정보(보호자·핀고정·삭제불가). 발작·알레르기·대처. 참고: docs/02 §3 JSONB(MED-004), docs/08-wbs.md §17.2.5</t>
         </is>
       </c>
+      <c r="J104" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="14" t="n">
@@ -5258,6 +5825,11 @@
           <t>MED-005 치료계획서(치료사). 목표·회기 계획·평가지표. 참고: docs/01 §2·§3, docs/02 §3 JSONB(MED-005), wireframes/web/59-therapist-plan.svg</t>
         </is>
       </c>
+      <c r="J105" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="n">
@@ -5301,6 +5873,11 @@
           <t>MED-006 치료 회기 일지(치료사). 회기 활동·반응·과제. 참고: docs/02 §3 JSONB(MED-006), wireframes/web/60-therapist-session-form.svg</t>
         </is>
       </c>
+      <c r="J106" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="14" t="n">
@@ -5344,6 +5921,11 @@
           <t>MED-007 치료 평가 보고서(치료사). 기간 성과·재평가. 참고: docs/02 §3 JSONB(MED-007), wireframes/web/61-therapist-evaluation.svg</t>
         </is>
       </c>
+      <c r="J107" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="14" t="n">
@@ -5387,6 +5969,11 @@
           <t>MED-008 정기 검진 요약(보호자). 참고: docs/02 §3 JSONB(MED-008)</t>
         </is>
       </c>
+      <c r="J108" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="14" t="n">
@@ -5430,6 +6017,11 @@
           <t>MED-009 치료 종결 평가(치료사·삭제불가, P1). 참고: docs/02 §3 JSONB(MED-009)</t>
         </is>
       </c>
+      <c r="J109" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="14" t="n">
@@ -5473,6 +6065,11 @@
           <t>MED-010 만성질환 관리(보호자, P1·중장년). 참고: docs/01 §6 중장년/노년기, docs/02 §3 JSONB(MED-010)</t>
         </is>
       </c>
+      <c r="J110" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="14" t="n">
@@ -5516,6 +6113,11 @@
           <t>EDU-001 IEP 개별화교육계획(특수교사·최대 공수). 현행수준·연간/단기목표·평가. 참고: docs/01 §2 아동기, docs/02 §3 JSONB(EDU-001), wireframes/web/45-teacher-iep-form.svg</t>
         </is>
       </c>
+      <c r="J111" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="14" t="n">
@@ -5559,6 +6161,11 @@
           <t>EDU-002 유아 특수교육 관찰(교사, P1·영유아). 참고: docs/01 §1, docs/02 §3 JSONB(EDU-002)</t>
         </is>
       </c>
+      <c r="J112" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="14" t="n">
@@ -5602,6 +6209,11 @@
           <t>EDU-003 IEP 중간 점검(교사). 목표 달성도 평가. 참고: docs/02 §3 JSONB(EDU-003), wireframes/web/46-teacher-iep-review.svg</t>
         </is>
       </c>
+      <c r="J113" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="14" t="n">
@@ -5645,6 +6257,11 @@
           <t>EDU-004 학교생활 관찰(교사). 참고: docs/02 §3 JSONB(EDU-004), wireframes/web/47-teacher-observation.svg</t>
         </is>
       </c>
+      <c r="J114" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="14" t="n">
@@ -5688,6 +6305,11 @@
           <t>EDU-005 통합교육 참여(교사, P1). 참고: docs/02 §3 JSONB(EDU-005)</t>
         </is>
       </c>
+      <c r="J115" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="14" t="n">
@@ -5731,6 +6353,11 @@
           <t>EDU-006 학교 치료지원(교사+치료사, P1). 참고: docs/02 §3 JSONB(EDU-006)</t>
         </is>
       </c>
+      <c r="J116" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="14" t="n">
@@ -5774,6 +6401,11 @@
           <t>EDU-007 전환교육 계획(교사·청소년). 진로·자립 준비. 참고: docs/01 §3 청소년기, docs/02 §3 JSONB(EDU-007), wireframes/web/48-teacher-transition.svg</t>
         </is>
       </c>
+      <c r="J117" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="14" t="n">
@@ -5817,6 +6449,11 @@
           <t>EDU-008 직업교육 참여(교사, P1). 참고: docs/02 §3 JSONB(EDU-008)</t>
         </is>
       </c>
+      <c r="J118" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="14" t="n">
@@ -5860,6 +6497,11 @@
           <t>EDU-009 졸업/수료(교사·삭제불가). 참고: docs/02 §3 JSONB(EDU-009)</t>
         </is>
       </c>
+      <c r="J119" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="n">
@@ -5903,6 +6545,11 @@
           <t>WEL-001 장애 등록(보호자·삭제불가). 장애유형·정도·등록일. 참고: docs/01 §1, docs/02 §3 JSONB(WEL-001)</t>
         </is>
       </c>
+      <c r="J120" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="14" t="n">
@@ -5946,6 +6593,11 @@
           <t>WEL-002 초기 복지 연계(복지사). 참고: docs/02 §3 JSONB(WEL-002)</t>
         </is>
       </c>
+      <c r="J121" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="n">
@@ -5989,6 +6641,11 @@
           <t>WEL-003 활동지원 계획서(복지사). 참고: docs/02 §3 JSONB(WEL-003)</t>
         </is>
       </c>
+      <c r="J122" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="14" t="n">
@@ -6032,6 +6689,11 @@
           <t>WEL-004 ISP 개별지원계획(복지사·최대 공수). 욕구·목표·서비스 매핑. 참고: docs/01 §5 성인기, docs/02 §3 JSONB(WEL-004), wireframes/web/53-worker-isp-form.svg</t>
         </is>
       </c>
+      <c r="J123" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="14" t="n">
@@ -6075,6 +6737,11 @@
           <t>WEL-005 ISP 중간 점검(복지사). 참고: docs/02 §3 JSONB(WEL-005), wireframes/web/52-worker-isp.svg</t>
         </is>
       </c>
+      <c r="J124" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="14" t="n">
@@ -6118,6 +6785,11 @@
           <t>WEL-006 서비스 이용 현황(복지사·매트릭스). 참고: docs/02 §3 JSONB(WEL-006), wireframes/web/55-worker-service-matrix.svg</t>
         </is>
       </c>
+      <c r="J125" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="14" t="n">
@@ -6161,6 +6833,11 @@
           <t>WEL-007 노인복지 연계(복지사, P2·노년). 참고: docs/01 §6, docs/02 §3 JSONB(WEL-007)</t>
         </is>
       </c>
+      <c r="J126" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="14" t="n">
@@ -6204,6 +6881,11 @@
           <t>DAI-001 영유아 돌봄(보호자, P1). 참고: docs/01 §1, docs/02 §3 JSONB(DAI-001)</t>
         </is>
       </c>
+      <c r="J127" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="14" t="n">
@@ -6247,6 +6929,11 @@
           <t>DAI-002 활동지원 일지(활동지원사·핵심). 활동·식사·특이사항. 참고: docs/04 §3 활동지원사, docs/02 §3 JSONB(DAI-002), wireframes/web/38-supporter-journal-form.svg</t>
         </is>
       </c>
+      <c r="J128" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="14" t="n">
@@ -6290,6 +6977,11 @@
           <t>DAI-003 행동 관찰(지원사). 참고: docs/02 §3 JSONB(DAI-003)</t>
         </is>
       </c>
+      <c r="J129" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="14" t="n">
@@ -6333,6 +7025,11 @@
           <t>DAI-004 식이 기록(지원사, P1). 참고: docs/02 §3 JSONB(DAI-004)</t>
         </is>
       </c>
+      <c r="J130" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="14" t="n">
@@ -6376,6 +7073,11 @@
           <t>DAI-005 수면 기록(지원사, P1). 참고: docs/02 §3 JSONB(DAI-005)</t>
         </is>
       </c>
+      <c r="J131" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="14" t="n">
@@ -6419,6 +7121,11 @@
           <t>TRA-001 전환계획서(복지사·성인전환기). 교육→자립 종합 계획. 참고: docs/01 §4 성인전환기, docs/02 §3 JSONB(TRA-001), wireframes/web/54-worker-transition.svg</t>
         </is>
       </c>
+      <c r="J132" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="14" t="n">
@@ -6462,6 +7169,11 @@
           <t>TRA-002 직업 역량 평가(복지사). 참고: docs/02 §3 JSONB(TRA-002)</t>
         </is>
       </c>
+      <c r="J133" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="14" t="n">
@@ -6505,6 +7217,11 @@
           <t>TRA-003 직업훈련/취업(복지사). 참고: docs/02 §3 JSONB(TRA-003)</t>
         </is>
       </c>
+      <c r="J134" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="14" t="n">
@@ -6548,6 +7265,11 @@
           <t>TRA-004 자립생활 계획(복지사, P1). 참고: docs/02 §3 JSONB(TRA-004)</t>
         </is>
       </c>
+      <c r="J135" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="14" t="n">
@@ -6591,6 +7313,11 @@
           <t>TRA-005 자립생활 경과(복지사, P1). 참고: docs/02 §3 JSONB(TRA-005)</t>
         </is>
       </c>
+      <c r="J136" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="14" t="n">
@@ -6634,6 +7361,11 @@
           <t>TRA-006 의사결정 지원(복지사+당사자, P1). 참고: docs/01 §5, docs/02 §3 JSONB(TRA-006)</t>
         </is>
       </c>
+      <c r="J137" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="14" t="n">
@@ -6677,6 +7409,11 @@
           <t>TRA-007 돌봄 전환 계획(복지사+보호자, P2·노년 대비). 참고: docs/01 §6, docs/02 §3 JSONB(TRA-007)</t>
         </is>
       </c>
+      <c r="J138" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="14" t="n">
@@ -6720,6 +7457,11 @@
           <t>LEG-001 장애인 증명서(보호자). 참고: docs/02 §3 JSONB(LEG-001)</t>
         </is>
       </c>
+      <c r="J139" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="14" t="n">
@@ -6763,6 +7505,11 @@
           <t>LEG-002 수급 기록(보호자). 참고: docs/02 §3 JSONB(LEG-002)</t>
         </is>
       </c>
+      <c r="J140" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="14" t="n">
@@ -6806,6 +7553,11 @@
           <t>LEG-003 후견 문서(보호자). 후견 유형·범위·기간. 참고: docs/01 §4·§5, docs/02 §3 JSONB(LEG-003)</t>
         </is>
       </c>
+      <c r="J141" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="14" t="n">
@@ -6849,6 +7601,11 @@
           <t>LEG-004 의사결정 지원 계약(보호자, P1). 참고: docs/02 §3 JSONB(LEG-004)</t>
         </is>
       </c>
+      <c r="J142" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="14" t="n">
@@ -6892,6 +7649,11 @@
           <t>LEG-005 노후 돌봄 문서(보호자, P2). 참고: docs/01 §6, docs/02 §3 JSONB(LEG-005)</t>
         </is>
       </c>
+      <c r="J143" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="15" t="n">
@@ -6935,6 +7697,11 @@
           <t>당사자 자기표현 입력 5스텝(기분·활동·사진·메모). 날짜별 1건. 참고: docs/06 §6 Flow-1 자기표현, docs/04 §2 당사자, docs/02 §3 JSONB(self_expression), wireframes/web/09-self-expression.svg</t>
         </is>
       </c>
+      <c r="J144" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="15" t="n">
@@ -6978,6 +7745,11 @@
           <t>특정 날짜 자기표현 단건 조회(오늘 기록 홈). 참고: wireframes/web/08-person-home.svg</t>
         </is>
       </c>
+      <c r="J145" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="15" t="n">
@@ -7021,6 +7793,11 @@
           <t>월·주 단위 자기표현 목록(캘린더/리스트). 참고: docs/02 §5 인덱스(date)</t>
         </is>
       </c>
+      <c r="J146" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="15" t="n">
@@ -7064,6 +7841,11 @@
           <t>자기표현 수정(작성 당일만 허용). 참고: docs/03 §RLS(self_expressions)</t>
         </is>
       </c>
+      <c r="J147" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="15" t="n">
@@ -7107,6 +7889,11 @@
           <t>자기표현 사진 업로드(presigned URL). 참고: docs/05 §5 파일 첨부</t>
         </is>
       </c>
+      <c r="J148" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="15" t="n">
@@ -7150,6 +7937,11 @@
           <t>자기표현 음성 메모 업로드(P1). 참고: docs/08-wbs.md §16.6.3</t>
         </is>
       </c>
+      <c r="J149" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="15" t="n">
@@ -7193,6 +7985,11 @@
           <t>자기표현 작성 시 보호자 요약 알림 발송. 참고: docs/05 §8 알림, notifications.self_expression_id FK</t>
         </is>
       </c>
+      <c r="J150" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="15" t="n">
@@ -7236,6 +8033,11 @@
           <t>연속 입력 일수 등 자기표현 통계(P1).</t>
         </is>
       </c>
+      <c r="J151" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="16" t="n">
@@ -7279,6 +8081,11 @@
           <t>Presigned URL 발급(업로드용). 참고: docs/05 §5 파일 첨부 프로세스, bkit:bkend-storage 스킬</t>
         </is>
       </c>
+      <c r="J152" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="16" t="n">
@@ -7322,6 +8129,11 @@
           <t>업로드 완료 후 record_files 메타데이터 등록. 참고: docs/02 §2(record_files)</t>
         </is>
       </c>
+      <c r="J153" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="16" t="n">
@@ -7365,6 +8177,11 @@
           <t>파일 단건 조회 + 다운로드 URL(CDN/presigned). 참고: bkit:bkend-storage 스킬</t>
         </is>
       </c>
+      <c r="J154" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="16" t="n">
@@ -7408,6 +8225,11 @@
           <t>특정 기록의 첨부 파일 목록.</t>
         </is>
       </c>
+      <c r="J155" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="16" t="n">
@@ -7451,6 +8273,11 @@
           <t>특정 자기표현의 첨부 파일 목록.</t>
         </is>
       </c>
+      <c r="J156" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="16" t="n">
@@ -7494,6 +8321,11 @@
           <t>파일 메타 수정(제목·민감도 sensitivity). 참고: docs/02 §4 Enum(sensitivity)</t>
         </is>
       </c>
+      <c r="J157" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="16" t="n">
@@ -7537,6 +8369,11 @@
           <t>파일 삭제(스토리지 객체 + 메타 동시).</t>
         </is>
       </c>
+      <c r="J158" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="16" t="n">
@@ -7580,6 +8417,11 @@
           <t>민감 파일(응급정보 등) 다운로드 시 추가 인증 미들웨어. 참고: docs/05 §11 보안 흐름, docs/08-wbs.md §17.2.5</t>
         </is>
       </c>
+      <c r="J159" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="16" t="n">
@@ -7623,6 +8465,11 @@
           <t>업로드 파일 바이러스 스캔 edge function(P2).</t>
         </is>
       </c>
+      <c r="J160" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="17" t="n">
@@ -7666,6 +8513,11 @@
           <t>이정표 추가(진단·입학·졸업·취업 등). category·event_date. 참고: docs/02 §2(life_milestones), docs/01-record-matrix.md</t>
         </is>
       </c>
+      <c r="J161" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="17" t="n">
@@ -7709,6 +8561,11 @@
           <t>이정표 단건 조회.</t>
         </is>
       </c>
+      <c r="J162" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="17" t="n">
@@ -7752,6 +8609,11 @@
           <t>당사자별 이정표 목록.</t>
         </is>
       </c>
+      <c r="J163" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="17" t="n">
@@ -7795,6 +8657,11 @@
           <t>이정표 수정.</t>
         </is>
       </c>
+      <c r="J164" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="17" t="n">
@@ -7838,6 +8705,11 @@
           <t>이정표 삭제.</t>
         </is>
       </c>
+      <c r="J165" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="17" t="n">
@@ -7881,6 +8753,11 @@
           <t>카테고리별 이정표 필터.</t>
         </is>
       </c>
+      <c r="J166" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="17" t="n">
@@ -7924,6 +8801,11 @@
           <t>records+milestones+self_expressions 통합 타임라인(시간 역순). 참고: docs/05 §6 생애주기 타임라인 조회, wireframes/web/03-timeline.svg</t>
         </is>
       </c>
+      <c r="J167" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="17" t="n">
@@ -7967,6 +8849,11 @@
           <t>타임라인 도메인 필터. 참고: docs/07 §1 도메인 컬러</t>
         </is>
       </c>
+      <c r="J168" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="17" t="n">
@@ -8010,6 +8897,11 @@
           <t>생애주기(life_stage)별 필터. 참고: docs/02 §4 Enum(life_stage)</t>
         </is>
       </c>
+      <c r="J169" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="17" t="n">
@@ -8053,6 +8945,11 @@
           <t>날짜 범위 필터.</t>
         </is>
       </c>
+      <c r="J170" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="17" t="n">
@@ -8096,6 +8993,11 @@
           <t>이정표만 필터링.</t>
         </is>
       </c>
+      <c r="J171" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="17" t="n">
@@ -8139,6 +9041,11 @@
           <t>작성자별 필터(P1).</t>
         </is>
       </c>
+      <c r="J172" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="17" t="n">
@@ -8182,6 +9089,11 @@
           <t>타임라인 PDF 내보내기(P1). 참고: docs/05 §6</t>
         </is>
       </c>
+      <c r="J173" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="17" t="n">
@@ -8225,6 +9137,11 @@
           <t>생애주기 전환 시 자동 마커 삽입 트리거. 참고: docs/05 §10 당사자 전환기 처리</t>
         </is>
       </c>
+      <c r="J174" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="18" t="n">
@@ -8268,6 +9185,11 @@
           <t>인수인계 생성 4스텝(분야·기간·요약·연계 기록). 참고: docs/06 §6 Flow-6 인수인계, docs/05 §7 인수인계, docs/02 §2(handovers), wireframes/web/56-worker-handover-create.svg</t>
         </is>
       </c>
+      <c r="J175" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="18" t="n">
@@ -8311,6 +9233,11 @@
           <t>인수인계 상세 조회(연계 기록 포함). 참고: wireframes/web/40-supporter-handover-detail.svg</t>
         </is>
       </c>
+      <c r="J176" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="18" t="n">
@@ -8354,6 +9281,11 @@
           <t>받은 인계 목록. 참고: wireframes/web/39-supporter-handover-list.svg</t>
         </is>
       </c>
+      <c r="J177" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="18" t="n">
@@ -8397,6 +9329,11 @@
           <t>전달한 인계 목록.</t>
         </is>
       </c>
+      <c r="J178" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="18" t="n">
@@ -8440,6 +9377,11 @@
           <t>인계 수정(미확인 상태에서만). 참고: docs/03 §RLS</t>
         </is>
       </c>
+      <c r="J179" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="18" t="n">
@@ -8483,6 +9425,11 @@
           <t>인계 삭제/취소(P1).</t>
         </is>
       </c>
+      <c r="J180" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="18" t="n">
@@ -8526,6 +9473,11 @@
           <t>Step1 — 분야·인계 기간·후임자 지정. 참고: docs/06 §6 Flow-6, wireframes/web/56-worker-handover-create.svg</t>
         </is>
       </c>
+      <c r="J181" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="18" t="n">
@@ -8569,6 +9521,11 @@
           <t>Step2 — 핵심 요약·특이사항 태그 작성.</t>
         </is>
       </c>
+      <c r="J182" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="18" t="n">
@@ -8612,6 +9569,11 @@
           <t>Step3 — 중요 기록 다중 선택(linked_record_ids).</t>
         </is>
       </c>
+      <c r="J183" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="18" t="n">
@@ -8655,6 +9617,11 @@
           <t>Step4 — 미리보기·발송 + 후임자 알림. 참고: docs/05 §8 알림</t>
         </is>
       </c>
+      <c r="J184" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="18" t="n">
@@ -8698,6 +9665,11 @@
           <t>후임자 인계 확인 처리(is_confirmed). 참고: docs/04 §3 활동지원사</t>
         </is>
       </c>
+      <c r="J185" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="18" t="n">
@@ -8741,6 +9713,11 @@
           <t>인계 확인 시 권한 자동 이양 트리거(옵션, P1). 참고: docs/05 §7·§2</t>
         </is>
       </c>
+      <c r="J186" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="19" t="n">
@@ -8784,6 +9761,11 @@
           <t>이벤트별 알림 자동 생성 트리거(기록 작성·권한 변경·인계 등). 참고: docs/05 §8 알림 발송/수신, docs/02 §3 JSONB(notification payload)</t>
         </is>
       </c>
+      <c r="J187" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="19" t="n">
@@ -8827,6 +9809,11 @@
           <t>알림 단건 조회.</t>
         </is>
       </c>
+      <c r="J188" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="19" t="n">
@@ -8870,6 +9857,11 @@
           <t>사용자별 알림 목록(페이징). 참고: wireframes/web/23-guardian-notifications.svg</t>
         </is>
       </c>
+      <c r="J189" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="19" t="n">
@@ -8913,6 +9905,11 @@
           <t>알림 읽음 처리.</t>
         </is>
       </c>
+      <c r="J190" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="19" t="n">
@@ -8956,6 +9953,11 @@
           <t>알림 일괄 읽음 처리.</t>
         </is>
       </c>
+      <c r="J191" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="19" t="n">
@@ -8999,6 +10001,11 @@
           <t>알림 삭제(P1).</t>
         </is>
       </c>
+      <c r="J192" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="19" t="n">
@@ -9042,6 +10049,11 @@
           <t>FCM 앱 푸시 발송 edge function. 참고: docs/05 §8, docs/08-wbs.md §16.6.1</t>
         </is>
       </c>
+      <c r="J193" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="19" t="n">
@@ -9085,6 +10097,11 @@
           <t>이메일 발송(SendGrid/Resend) edge function. 참고: docs/05 §8</t>
         </is>
       </c>
+      <c r="J194" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="19" t="n">
@@ -9128,6 +10145,11 @@
           <t>SMS 발송(응급용, P1).</t>
         </is>
       </c>
+      <c r="J195" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="19" t="n">
@@ -9171,6 +10193,11 @@
           <t>사용자별 알림 채널 설정 조회. 참고: wireframes/web/27-guardian-notification-settings.svg</t>
         </is>
       </c>
+      <c r="J196" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="19" t="n">
@@ -9214,6 +10241,11 @@
           <t>알림 채널 설정 수정.</t>
         </is>
       </c>
+      <c r="J197" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="19" t="n">
@@ -9257,6 +10289,11 @@
           <t>알림 유형별 on/off 토글 매트릭스. 참고: wireframes/web/27-guardian-notification-settings.svg</t>
         </is>
       </c>
+      <c r="J198" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="19" t="n">
@@ -9300,6 +10337,11 @@
           <t>방해 금지 시간대 설정(P1).</t>
         </is>
       </c>
+      <c r="J199" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="19" t="n">
@@ -9343,6 +10385,11 @@
           <t>앱 설치 시 푸시 토큰 등록. 참고: docs/08-wbs.md §16.6.1</t>
         </is>
       </c>
+      <c r="J200" s="39" t="inlineStr">
+        <is>
+          <t>개발자 B</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="20" t="n">
@@ -9386,6 +10433,11 @@
           <t>모든 read 자동 로깅 트리거(누가 무엇을 열람). 참고: docs/02 §2(access_logs), docs/05 §9 접근 로그 조회</t>
         </is>
       </c>
+      <c r="J201" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="20" t="n">
@@ -9429,6 +10481,11 @@
           <t>모든 write 자동 로깅 트리거. 참고: docs/03 §RLS</t>
         </is>
       </c>
+      <c r="J202" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="20" t="n">
@@ -9472,6 +10529,11 @@
           <t>권한 외 접근 시도 별도 로깅. 참고: docs/05 §11 보안 흐름</t>
         </is>
       </c>
+      <c r="J203" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="20" t="n">
@@ -9515,6 +10577,11 @@
           <t>당사자별 접근 로그 조회(보호자 투명성). 참고: docs/05 §9, wireframes/web/22-guardian-access-log.svg</t>
         </is>
       </c>
+      <c r="J204" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="20" t="n">
@@ -9558,6 +10625,11 @@
           <t>접근 로그 필터(날짜·접근자·동작).</t>
         </is>
       </c>
+      <c r="J205" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="20" t="n">
@@ -9601,6 +10673,11 @@
           <t>이상 활동 자동 감지 rule engine(P1). 참고: docs/05 §11</t>
         </is>
       </c>
+      <c r="J206" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="20" t="n">
@@ -9644,6 +10721,11 @@
           <t>접근 로그 CSV 내보내기.</t>
         </is>
       </c>
+      <c r="J207" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="20" t="n">
@@ -9687,6 +10769,11 @@
           <t>월간 접근 보고서 자동 발송 cron(P1).</t>
         </is>
       </c>
+      <c r="J208" s="38" t="inlineStr">
+        <is>
+          <t>개발자 A</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="21" t="n">
@@ -9730,6 +10817,11 @@
           <t>컬러 토큰(Primary·6 도메인 컬러·Status). 참고: docs/07-design-system.md §1 컬러 시스템, §10 Tailwind 설정</t>
         </is>
       </c>
+      <c r="J209" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="21" t="n">
@@ -9773,6 +10865,11 @@
           <t>타이포 토큰(Pretendard 스케일). 참고: docs/07 §2 타이포그래피</t>
         </is>
       </c>
+      <c r="J210" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="21" t="n">
@@ -9816,6 +10913,11 @@
           <t>스페이싱·보더 레디어스·엘리베이션 토큰. 참고: docs/07 §3·§4·§5</t>
         </is>
       </c>
+      <c r="J211" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="21" t="n">
@@ -9859,6 +10961,11 @@
           <t>당사자 접근성 토큰(큰 글씨·고대비). 참고: docs/07 §9 당사자 접근성 모드</t>
         </is>
       </c>
+      <c r="J212" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="21" t="n">
@@ -9902,6 +11009,11 @@
           <t>Button(primary/secondary/destructive). 참고: docs/07 §8 컴포넌트 라이브러리(Button)</t>
         </is>
       </c>
+      <c r="J213" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="21" t="n">
@@ -9945,6 +11057,11 @@
           <t>Input(text/email/password/number). 참고: docs/07 §8(Input)</t>
         </is>
       </c>
+      <c r="J214" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="21" t="n">
@@ -9988,6 +11105,11 @@
           <t>TextArea. 참고: docs/07 §8</t>
         </is>
       </c>
+      <c r="J215" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="21" t="n">
@@ -10031,6 +11153,11 @@
           <t>Select/Dropdown. 참고: docs/07 §8</t>
         </is>
       </c>
+      <c r="J216" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="21" t="n">
@@ -10074,6 +11201,11 @@
           <t>Checkbox/Radio. 참고: docs/07 §8</t>
         </is>
       </c>
+      <c r="J217" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="21" t="n">
@@ -10117,6 +11249,11 @@
           <t>Toggle/Switch. 참고: docs/07 §8</t>
         </is>
       </c>
+      <c r="J218" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="21" t="n">
@@ -10160,6 +11297,11 @@
           <t>Badge(도메인 6 컬러 variant). 참고: docs/07 §1 도메인 컬러·§8</t>
         </is>
       </c>
+      <c r="J219" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="21" t="n">
@@ -10203,6 +11345,11 @@
           <t>Avatar. 참고: docs/07 §8</t>
         </is>
       </c>
+      <c r="J220" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="21" t="n">
@@ -10246,6 +11393,11 @@
           <t>RecordCard(도메인 컬러+첨부 미리보기). 참고: docs/07 §8 컴포넌트 라이브러리(RecordCard)</t>
         </is>
       </c>
+      <c r="J221" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="21" t="n">
@@ -10289,6 +11441,11 @@
           <t>PersonCard(당사자 카드). 참고: docs/07 §8</t>
         </is>
       </c>
+      <c r="J222" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="21" t="n">
@@ -10332,6 +11489,11 @@
           <t>NotificationCard(3 type variant). 참고: docs/07 §8</t>
         </is>
       </c>
+      <c r="J223" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="21" t="n">
@@ -10375,6 +11537,11 @@
           <t>IconSelectorCard(자기표현 전용, 큰 아이콘). 참고: docs/07 §6 아이콘·§9, docs/06 §6 Flow-1</t>
         </is>
       </c>
+      <c r="J224" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="21" t="n">
@@ -10418,6 +11585,11 @@
           <t>StepIndicator(위자드 진행 표시). 참고: docs/07 §8, docs/06 §6 플로우</t>
         </is>
       </c>
+      <c r="J225" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="21" t="n">
@@ -10461,6 +11633,11 @@
           <t>웹 Sidebar(240px↔64px 접힘). 참고: docs/06 §2 내비게이션 패턴, docs/07 §8</t>
         </is>
       </c>
+      <c r="J226" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="21" t="n">
@@ -10504,6 +11681,11 @@
           <t>웹 GlobalHeader(검색·알림·프로필). 참고: docs/06 §4 반응형 웹 IA</t>
         </is>
       </c>
+      <c r="J227" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="21" t="n">
@@ -10547,6 +11729,11 @@
           <t>모바일 BottomTabBar(역할별 variant). 참고: docs/06 §5 모바일 앱 IA, §2 내비게이션</t>
         </is>
       </c>
+      <c r="J228" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="21" t="n">
@@ -10590,6 +11777,11 @@
           <t>모바일 NavigationBar(Push 스택용). 참고: docs/06 §5</t>
         </is>
       </c>
+      <c r="J229" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="22" t="n">
@@ -10633,6 +11825,11 @@
           <t>보호자 로그인 화면(이메일·소셜). 참고: docs/06 §4 반응형 웹 IA, wireframes/web/01-login.svg</t>
         </is>
       </c>
+      <c r="J230" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="22" t="n">
@@ -10676,6 +11873,11 @@
           <t>회원가입 역할 선택. 참고: docs/05 §1 온보딩, wireframes/web/11-signup-role.svg</t>
         </is>
       </c>
+      <c r="J231" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="22" t="n">
@@ -10719,6 +11921,11 @@
           <t>회원가입 기본정보 입력. 참고: wireframes/web/12-signup-profile.svg</t>
         </is>
       </c>
+      <c r="J232" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="22" t="n">
@@ -10762,6 +11969,11 @@
           <t>이메일 인증 화면. 참고: wireframes/web/13-signup-verify.svg</t>
         </is>
       </c>
+      <c r="J233" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="22" t="n">
@@ -10805,6 +12017,11 @@
           <t>초대 링크 수락 화면. 참고: docs/05 §1, wireframes/web/14-invite-accept.svg</t>
         </is>
       </c>
+      <c r="J234" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="22" t="n">
@@ -10848,6 +12065,11 @@
           <t>비밀번호 재설정 화면. 참고: wireframes/web/15-reset-password.svg</t>
         </is>
       </c>
+      <c r="J235" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="22" t="n">
@@ -10891,6 +12113,11 @@
           <t>보호자 대시보드(당사자 목록·최근 활동·알림). 참고: docs/04 §1 보호자, wireframes/web/02-guardian-dashboard.svg</t>
         </is>
       </c>
+      <c r="J236" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="22" t="n">
@@ -10934,6 +12161,11 @@
           <t>당사자 프로필(요약·권한 현황). 참고: wireframes/web/16-guardian-person-profile.svg</t>
         </is>
       </c>
+      <c r="J237" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="22" t="n">
@@ -10977,6 +12209,11 @@
           <t>당사자 등록 위자드 5스텝. 참고: docs/04 §1, wireframes/web/17-guardian-person-register.svg</t>
         </is>
       </c>
+      <c r="J238" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="22" t="n">
@@ -11020,6 +12257,11 @@
           <t>생애주기 타임라인. 참고: docs/05 §6, wireframes/web/03-timeline.svg</t>
         </is>
       </c>
+      <c r="J239" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="22" t="n">
@@ -11063,6 +12305,11 @@
           <t>전체 기록 관리. 참고: wireframes/web/04-record-list.svg</t>
         </is>
       </c>
+      <c r="J240" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="22" t="n">
@@ -11106,6 +12353,11 @@
           <t>도메인별 기록 목록. 참고: wireframes/web/18-guardian-records-domain.svg</t>
         </is>
       </c>
+      <c r="J241" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="22" t="n">
@@ -11149,6 +12401,11 @@
           <t>기록 상세(Split 뷰). 참고: wireframes/web/05-record-detail.svg</t>
         </is>
       </c>
+      <c r="J242" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="22" t="n">
@@ -11192,6 +12449,11 @@
           <t>기록 작성 위자드 5스텝(도메인별 분기). 참고: docs/05 §4 기록 작성 공통, wireframes/web/06-record-form.svg</t>
         </is>
       </c>
+      <c r="J243" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="22" t="n">
@@ -11235,6 +12497,11 @@
           <t>기록 수정. 참고: wireframes/web/19-guardian-record-edit.svg</t>
         </is>
       </c>
+      <c r="J244" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="22" t="n">
@@ -11278,6 +12545,11 @@
           <t>권한 매트릭스(이해관계자×도메인). 참고: wireframes/web/07-permission-matrix.svg</t>
         </is>
       </c>
+      <c r="J245" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="22" t="n">
@@ -11321,6 +12593,11 @@
           <t>이해관계자 상세(받은 권한·이력). 참고: wireframes/web/20-guardian-stakeholder-detail.svg</t>
         </is>
       </c>
+      <c r="J246" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="22" t="n">
@@ -11364,6 +12641,11 @@
           <t>권한 부여 위자드 4스텝. 참고: docs/06 §6, wireframes/web/21-guardian-grant-wizard.svg</t>
         </is>
       </c>
+      <c r="J247" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="22" t="n">
@@ -11407,6 +12689,11 @@
           <t>권한 수정·회수 모달. 참고: wireframes/web/28-guardian-permission-modals.svg</t>
         </is>
       </c>
+      <c r="J248" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="22" t="n">
@@ -11450,6 +12737,11 @@
           <t>접근 로그 화면. 참고: docs/05 §9, wireframes/web/22-guardian-access-log.svg</t>
         </is>
       </c>
+      <c r="J249" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="22" t="n">
@@ -11493,6 +12785,11 @@
           <t>알림 목록. 참고: wireframes/web/23-guardian-notifications.svg</t>
         </is>
       </c>
+      <c r="J250" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="22" t="n">
@@ -11536,6 +12833,11 @@
           <t>설정 허브. 참고: wireframes/web/10-settings.svg</t>
         </is>
       </c>
+      <c r="J251" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="22" t="n">
@@ -11579,6 +12881,11 @@
           <t>프로필 편집. 참고: wireframes/web/24-guardian-profile-edit.svg</t>
         </is>
       </c>
+      <c r="J252" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="22" t="n">
@@ -11622,6 +12929,11 @@
           <t>당사자 정보 편집. 참고: wireframes/web/25-guardian-person-edit.svg</t>
         </is>
       </c>
+      <c r="J253" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="22" t="n">
@@ -11665,6 +12977,11 @@
           <t>응급 정보 편집(추가 인증). 참고: wireframes/web/26-guardian-emergency-edit.svg</t>
         </is>
       </c>
+      <c r="J254" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="22" t="n">
@@ -11708,6 +13025,11 @@
           <t>알림 설정. 참고: wireframes/web/27-guardian-notification-settings.svg</t>
         </is>
       </c>
+      <c r="J255" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="23" t="n">
@@ -11751,6 +13073,11 @@
           <t>당사자 오늘 기록 홈(큰 CTA). 참고: docs/04 §2 당사자, docs/07 §9, wireframes/web/08-person-home.svg</t>
         </is>
       </c>
+      <c r="J256" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="23" t="n">
@@ -11794,6 +13121,11 @@
           <t>자기표현 위자드(Flow-1, 아이콘 기반). 참고: docs/06 §6 Flow-1, wireframes/web/09-self-expression.svg</t>
         </is>
       </c>
+      <c r="J257" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="23" t="n">
@@ -11837,6 +13169,11 @@
           <t>자기표현 완료 애니메이션(긍정 피드백). 참고: docs/07 §7 모션 &amp; 애니메이션</t>
         </is>
       </c>
+      <c r="J258" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="23" t="n">
@@ -11880,6 +13217,11 @@
           <t>내 기록 분야 그리드. 참고: wireframes/web/29-person-records.svg</t>
         </is>
       </c>
+      <c r="J259" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="23" t="n">
@@ -11923,6 +13265,11 @@
           <t>기록 상세(쉬운 요약 summary 필드). 참고: wireframes/web/30-person-record-detail.svg</t>
         </is>
       </c>
+      <c r="J260" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="23" t="n">
@@ -11966,6 +13313,11 @@
           <t>설정 허브(큰 카드). 참고: wireframes/web/31-person-settings.svg</t>
         </is>
       </c>
+      <c r="J261" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="23" t="n">
@@ -12009,6 +13361,11 @@
           <t>접근성 설정(글씨·대비·TTS). 참고: docs/07 §9, wireframes/web/32-person-accessibility.svg</t>
         </is>
       </c>
+      <c r="J262" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="23" t="n">
@@ -12052,6 +13409,11 @@
           <t>내 정보. 참고: wireframes/web/33-person-profile.svg</t>
         </is>
       </c>
+      <c r="J263" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="23" t="n">
@@ -12095,6 +13457,11 @@
           <t>알림(큰 카드). 참고: wireframes/web/34-person-notifications.svg</t>
         </is>
       </c>
+      <c r="J264" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="23" t="n">
@@ -12138,6 +13505,11 @@
           <t>접근성 모드 자동 적용(theme switch). 참고: docs/07 §9 당사자 접근성 모드, tokens-a11y</t>
         </is>
       </c>
+      <c r="J265" s="40" t="inlineStr">
+        <is>
+          <t>개발자 C</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="24" t="n">
@@ -12181,6 +13553,11 @@
           <t>활동지원사 홈. 참고: docs/04 §3 활동지원사, wireframes/web/35-supporter-home.svg</t>
         </is>
       </c>
+      <c r="J266" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="24" t="n">
@@ -12224,6 +13601,11 @@
           <t>일지 목록. 참고: wireframes/web/36-supporter-journal-list.svg</t>
         </is>
       </c>
+      <c r="J267" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="24" t="n">
@@ -12267,6 +13649,11 @@
           <t>일지 상세. 참고: wireframes/web/37-supporter-journal-detail.svg</t>
         </is>
       </c>
+      <c r="J268" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="24" t="n">
@@ -12310,6 +13697,11 @@
           <t>일지 작성 위자드 5스텝(Flow-4). 참고: docs/06 §6 Flow-4, wireframes/web/38-supporter-journal-form.svg</t>
         </is>
       </c>
+      <c r="J269" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="24" t="n">
@@ -12353,6 +13745,11 @@
           <t>일지 수정. 참고: wireframes/web/38-supporter-journal-form.svg</t>
         </is>
       </c>
+      <c r="J270" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="24" t="n">
@@ -12396,6 +13793,11 @@
           <t>인수인계 목록. 참고: wireframes/web/39-supporter-handover-list.svg</t>
         </is>
       </c>
+      <c r="J271" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="24" t="n">
@@ -12439,6 +13841,11 @@
           <t>인수인계 상세(확인 처리). 참고: docs/05 §7, wireframes/web/40-supporter-handover-detail.svg</t>
         </is>
       </c>
+      <c r="J272" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="24" t="n">
@@ -12482,6 +13889,11 @@
           <t>알림+설정 통합. 참고: wireframes/web/41-supporter-notifications-settings.svg</t>
         </is>
       </c>
+      <c r="J273" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="24" t="n">
@@ -12525,6 +13937,11 @@
           <t>교사 홈(담당 학생). 참고: docs/04 §4 특수교사, wireframes/web/42-teacher-home.svg</t>
         </is>
       </c>
+      <c r="J274" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="24" t="n">
@@ -12568,6 +13985,11 @@
           <t>IEP 목록. 참고: wireframes/web/43-teacher-iep-list.svg</t>
         </is>
       </c>
+      <c r="J275" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="24" t="n">
@@ -12611,6 +14033,11 @@
           <t>IEP 상세. 참고: wireframes/web/44-teacher-iep-detail.svg</t>
         </is>
       </c>
+      <c r="J276" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="24" t="n">
@@ -12654,6 +14081,11 @@
           <t>IEP 작성 위자드 6스텝(Flow-5·최대 공수). 참고: docs/06 §6 Flow-5, docs/02 §3 JSONB(EDU-001), wireframes/web/45-teacher-iep-form.svg</t>
         </is>
       </c>
+      <c r="J277" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="24" t="n">
@@ -12697,6 +14129,11 @@
           <t>IEP 중간 점검. 참고: wireframes/web/46-teacher-iep-review.svg</t>
         </is>
       </c>
+      <c r="J278" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="24" t="n">
@@ -12740,6 +14177,11 @@
           <t>관찰 기록 목록. 참고: wireframes/web/47-teacher-observation.svg</t>
         </is>
       </c>
+      <c r="J279" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="24" t="n">
@@ -12783,6 +14225,11 @@
           <t>관찰 기록 작성. 참고: wireframes/web/47-teacher-observation.svg</t>
         </is>
       </c>
+      <c r="J280" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="24" t="n">
@@ -12826,6 +14273,11 @@
           <t>전환교육 목록. 참고: wireframes/web/48-teacher-transition.svg</t>
         </is>
       </c>
+      <c r="J281" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="24" t="n">
@@ -12869,6 +14321,11 @@
           <t>전환교육 작성 4스텝. 참고: wireframes/web/48-teacher-transition.svg</t>
         </is>
       </c>
+      <c r="J282" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="24" t="n">
@@ -12912,6 +14369,11 @@
           <t>교육 타임라인(도메인 필터). 참고: wireframes/web/49-teacher-timeline.svg</t>
         </is>
       </c>
+      <c r="J283" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="24" t="n">
@@ -12955,6 +14417,11 @@
           <t>알림+설정. 참고: wireframes/web/50-teacher-notifications-settings.svg</t>
         </is>
       </c>
+      <c r="J284" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="24" t="n">
@@ -12998,6 +14465,11 @@
           <t>복지사 홈. 참고: docs/04 §5 사회복지사, wireframes/web/51-worker-home.svg</t>
         </is>
       </c>
+      <c r="J285" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="24" t="n">
@@ -13041,6 +14513,11 @@
           <t>ISP 목록. 참고: wireframes/web/52-worker-isp.svg</t>
         </is>
       </c>
+      <c r="J286" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="24" t="n">
@@ -13084,6 +14561,11 @@
           <t>ISP 상세. 참고: wireframes/web/52-worker-isp.svg</t>
         </is>
       </c>
+      <c r="J287" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="24" t="n">
@@ -13127,6 +14609,11 @@
           <t>ISP 작성 위자드 5스텝(최대 공수). 참고: docs/02 §3 JSONB(WEL-004), wireframes/web/53-worker-isp-form.svg</t>
         </is>
       </c>
+      <c r="J288" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="24" t="n">
@@ -13170,6 +14657,11 @@
           <t>ISP 중간 점검. 참고: wireframes/web/52-worker-isp.svg</t>
         </is>
       </c>
+      <c r="J289" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="24" t="n">
@@ -13213,6 +14705,11 @@
           <t>전환계획 목록. 참고: wireframes/web/54-worker-transition.svg</t>
         </is>
       </c>
+      <c r="J290" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="24" t="n">
@@ -13256,6 +14753,11 @@
           <t>전환계획 작성 5스텝(최대 공수). 참고: docs/02 §3 JSONB(TRA-001), wireframes/web/54-worker-transition.svg</t>
         </is>
       </c>
+      <c r="J291" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="24" t="n">
@@ -13299,6 +14801,11 @@
           <t>서비스 이용 현황 매트릭스. 참고: wireframes/web/55-worker-service-matrix.svg</t>
         </is>
       </c>
+      <c r="J292" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="24" t="n">
@@ -13342,6 +14849,11 @@
           <t>복지+전환 타임라인.</t>
         </is>
       </c>
+      <c r="J293" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="24" t="n">
@@ -13385,6 +14897,11 @@
           <t>인수인계 목록.</t>
         </is>
       </c>
+      <c r="J294" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="24" t="n">
@@ -13428,6 +14945,11 @@
           <t>인수인계 생성 4스텝(Flow-6). 참고: docs/06 §6 Flow-6, wireframes/web/56-worker-handover-create.svg</t>
         </is>
       </c>
+      <c r="J295" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="24" t="n">
@@ -13471,6 +14993,11 @@
           <t>알림+설정. 참고: wireframes/web/57-worker-notifications-settings.svg</t>
         </is>
       </c>
+      <c r="J296" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="24" t="n">
@@ -13514,6 +15041,11 @@
           <t>치료사 홈(오늘 회기). 참고: docs/04 §6 치료사, wireframes/web/58-therapist-home.svg</t>
         </is>
       </c>
+      <c r="J297" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="24" t="n">
@@ -13557,6 +15089,11 @@
           <t>치료계획서 목록. 참고: wireframes/web/59-therapist-plan.svg</t>
         </is>
       </c>
+      <c r="J298" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="24" t="n">
@@ -13600,6 +15137,11 @@
           <t>치료계획서 상세. 참고: wireframes/web/59-therapist-plan.svg</t>
         </is>
       </c>
+      <c r="J299" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="24" t="n">
@@ -13643,6 +15185,11 @@
           <t>치료계획서 작성 5스텝. 참고: docs/02 §3 JSONB(MED-005), wireframes/web/59-therapist-plan.svg</t>
         </is>
       </c>
+      <c r="J300" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="24" t="n">
@@ -13686,6 +15233,11 @@
           <t>회기 일지 목록. 참고: wireframes/web/60-therapist-session-form.svg</t>
         </is>
       </c>
+      <c r="J301" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="24" t="n">
@@ -13729,6 +15281,11 @@
           <t>회기 일지 작성. 참고: docs/02 §3 JSONB(MED-006), wireframes/web/60-therapist-session-form.svg</t>
         </is>
       </c>
+      <c r="J302" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="24" t="n">
@@ -13772,6 +15329,11 @@
           <t>평가 보고서 목록. 참고: wireframes/web/61-therapist-evaluation.svg</t>
         </is>
       </c>
+      <c r="J303" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="24" t="n">
@@ -13815,6 +15377,11 @@
           <t>평가 보고서 작성 4스텝. 참고: docs/02 §3 JSONB(MED-007), wireframes/web/61-therapist-evaluation.svg</t>
         </is>
       </c>
+      <c r="J304" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="24" t="n">
@@ -13858,6 +15425,11 @@
           <t>의료 타임라인. 참고: wireframes/web/62-therapist-timeline-settings.svg</t>
         </is>
       </c>
+      <c r="J305" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="24" t="n">
@@ -13901,6 +15473,11 @@
           <t>알림+설정. 참고: wireframes/web/62-therapist-timeline-settings.svg</t>
         </is>
       </c>
+      <c r="J306" s="41" t="inlineStr">
+        <is>
+          <t>개발자 D</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="10" t="n">
@@ -13944,6 +15521,11 @@
           <t>모바일 로그인. 참고: docs/06 §5 모바일 앱 IA, wireframes/mobile/01-m-login.svg</t>
         </is>
       </c>
+      <c r="J307" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="10" t="n">
@@ -13987,6 +15569,11 @@
           <t>회원가입 역할 선택. 참고: wireframes/mobile/06-m-signup-role.svg</t>
         </is>
       </c>
+      <c r="J308" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="10" t="n">
@@ -14030,6 +15617,11 @@
           <t>회원가입·이메일 인증·재설정 통합 플로우. 참고: docs/05 §1 온보딩</t>
         </is>
       </c>
+      <c r="J309" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="10" t="n">
@@ -14073,6 +15665,11 @@
           <t>초대 수락(Deep Link 처리). 참고: docs/08-wbs.md §16.6.6</t>
         </is>
       </c>
+      <c r="J310" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="10" t="n">
@@ -14116,6 +15713,11 @@
           <t>보호자 홈(Bottom Tab). 참고: wireframes/mobile/02-m-guardian-home.svg</t>
         </is>
       </c>
+      <c r="J311" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="10" t="n">
@@ -14159,6 +15761,11 @@
           <t>타임라인. 참고: wireframes/mobile/03-m-timeline.svg</t>
         </is>
       </c>
+      <c r="J312" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="10" t="n">
@@ -14202,6 +15809,11 @@
           <t>기록 상세(Push). 참고: wireframes/mobile/07-m-record-detail.svg</t>
         </is>
       </c>
+      <c r="J313" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="10" t="n">
@@ -14245,6 +15857,11 @@
           <t>기록 작성(Full-screen Flow). 참고: wireframes/mobile/08-m-record-form.svg</t>
         </is>
       </c>
+      <c r="J314" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="10" t="n">
@@ -14288,6 +15905,11 @@
           <t>권한 매트릭스(카드 리스트). 참고: wireframes/mobile/09-m-permissions.svg</t>
         </is>
       </c>
+      <c r="J315" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="10" t="n">
@@ -14331,6 +15953,11 @@
           <t>권한 부여 위자드. 참고: wireframes/mobile/10-m-grant-wizard.svg</t>
         </is>
       </c>
+      <c r="J316" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="10" t="n">
@@ -14374,6 +16001,11 @@
           <t>알림(인라인 액션). 참고: wireframes/mobile/11-m-notifications.svg</t>
         </is>
       </c>
+      <c r="J317" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="10" t="n">
@@ -14417,6 +16049,11 @@
           <t>설정(당사자별 진입). 참고: wireframes/mobile/12-m-settings.svg</t>
         </is>
       </c>
+      <c r="J318" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="10" t="n">
@@ -14460,6 +16097,11 @@
           <t>당사자 오늘 기록 홈(큰 CTA). 참고: docs/07 §9 접근성, wireframes/mobile/04-m-person-home.svg</t>
         </is>
       </c>
+      <c r="J319" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="10" t="n">
@@ -14503,6 +16145,11 @@
           <t>자기표현 위자드 4스텝(풀스크린). 참고: docs/06 §6 Flow-1, wireframes/mobile/05-m-self-expression.svg</t>
         </is>
       </c>
+      <c r="J320" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="10" t="n">
@@ -14546,6 +16193,11 @@
           <t>내 기록(분야 그리드). 참고: wireframes/mobile/13-m-person-records.svg</t>
         </is>
       </c>
+      <c r="J321" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="10" t="n">
@@ -14589,6 +16241,11 @@
           <t>기록 상세(쉬운 요약). 참고: wireframes/mobile/14-m-person-record-detail.svg</t>
         </is>
       </c>
+      <c r="J322" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="10" t="n">
@@ -14632,6 +16289,11 @@
           <t>설정(큰 카드). 참고: wireframes/mobile/15-m-person-settings.svg</t>
         </is>
       </c>
+      <c r="J323" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="10" t="n">
@@ -14675,6 +16337,11 @@
           <t>활동지원사 홈(대형 일지 CTA). 참고: wireframes/mobile/16-m-supporter-home.svg</t>
         </is>
       </c>
+      <c r="J324" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="10" t="n">
@@ -14718,6 +16385,11 @@
           <t>일지 작성 위자드 5스텝. 참고: wireframes/mobile/17-m-supporter-journal-form.svg</t>
         </is>
       </c>
+      <c r="J325" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="10" t="n">
@@ -14761,6 +16433,11 @@
           <t>인수인계 목록. 참고: wireframes/mobile/18-m-supporter-handover.svg</t>
         </is>
       </c>
+      <c r="J326" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="10" t="n">
@@ -14804,6 +16481,11 @@
           <t>교사 홈. 참고: wireframes/mobile/19-m-teacher-home.svg</t>
         </is>
       </c>
+      <c r="J327" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="10" t="n">
@@ -14847,6 +16529,11 @@
           <t>IEP 상세. 참고: wireframes/mobile/20-m-teacher-iep-detail.svg</t>
         </is>
       </c>
+      <c r="J328" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="10" t="n">
@@ -14890,6 +16577,11 @@
           <t>복지사 홈. 참고: wireframes/mobile/21-m-worker-home.svg</t>
         </is>
       </c>
+      <c r="J329" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="10" t="n">
@@ -14933,6 +16625,11 @@
           <t>ISP 상세. 참고: wireframes/mobile/22-m-worker-isp-detail.svg</t>
         </is>
       </c>
+      <c r="J330" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="10" t="n">
@@ -14976,6 +16673,11 @@
           <t>치료사 홈. 참고: wireframes/mobile/23-m-therapist-home.svg</t>
         </is>
       </c>
+      <c r="J331" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="10" t="n">
@@ -15019,6 +16721,11 @@
           <t>회기 일지 작성. 참고: wireframes/mobile/24-m-therapist-session.svg</t>
         </is>
       </c>
+      <c r="J332" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="10" t="n">
@@ -15062,6 +16769,11 @@
           <t>FCM 푸시 알림 통합(토큰 등록·수신). 참고: docs/05 §8 알림, docs/08-wbs.md §10.2.1·§10.2.8</t>
         </is>
       </c>
+      <c r="J333" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="10" t="n">
@@ -15105,6 +16817,11 @@
           <t>카메라/갤러리 사진 첨부. 참고: docs/05 §5 파일 첨부</t>
         </is>
       </c>
+      <c r="J334" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="10" t="n">
@@ -15148,6 +16865,11 @@
           <t>음성 메모 녹음(P1). 참고: docs/08-wbs.md §6.6</t>
         </is>
       </c>
+      <c r="J335" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="10" t="n">
@@ -15191,6 +16913,11 @@
           <t>일지 오프라인 임시저장(AsyncStorage) 후 동기화. 참고: docs/04 §3 활동지원사</t>
         </is>
       </c>
+      <c r="J336" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="10" t="n">
@@ -15234,6 +16961,11 @@
           <t>생체 인증(Face ID/지문) — 민감정보 보호. 참고: docs/08-wbs.md §17.2.5</t>
         </is>
       </c>
+      <c r="J337" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="10" t="n">
@@ -15277,6 +17009,11 @@
           <t>Deep Link 라우팅(초대·알림 진입). 참고: docs/08-wbs.md §16.1.4</t>
         </is>
       </c>
+      <c r="J338" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="10" t="n">
@@ -15320,6 +17057,11 @@
           <t>OTA 업데이트(Expo Updates, P1).</t>
         </is>
       </c>
+      <c r="J339" s="42" t="inlineStr">
+        <is>
+          <t>개발자 E</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="25" t="n">
@@ -15363,6 +17105,11 @@
           <t>랜딩 페이지 메타 태그(P1).</t>
         </is>
       </c>
+      <c r="J340" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="25" t="n">
@@ -15406,6 +17153,11 @@
           <t>Sitemap·robots.txt(P1).</t>
         </is>
       </c>
+      <c r="J341" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="25" t="n">
@@ -15449,6 +17201,11 @@
           <t>OG 이미지·소셜 미리보기(P2).</t>
         </is>
       </c>
+      <c r="J342" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="25" t="n">
@@ -15492,6 +17249,11 @@
           <t>OWASP Top 10 자체 점검. 참고: docs/05 §11 시스템 보안 흐름, bkit:phase-7-seo-security 스킬</t>
         </is>
       </c>
+      <c r="J343" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="25" t="n">
@@ -15535,6 +17297,11 @@
           <t>XSS 방어 — 입력값 sanitize.</t>
         </is>
       </c>
+      <c r="J344" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="25" t="n">
@@ -15578,6 +17345,11 @@
           <t>CSRF 토큰 적용.</t>
         </is>
       </c>
+      <c r="J345" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="25" t="n">
@@ -15621,6 +17393,11 @@
           <t>SQL Injection 방어 검증(RLS + Prisma 파라미터화). 참고: docs/03 §RLS</t>
         </is>
       </c>
+      <c r="J346" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="25" t="n">
@@ -15664,6 +17441,11 @@
           <t>응급정보 접근 시 PIN/생체 추가 인증. 참고: docs/05 §11, docs/02 §3 JSONB(emergency)</t>
         </is>
       </c>
+      <c r="J347" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="25" t="n">
@@ -15707,6 +17489,11 @@
           <t>민감 파일 다운로드 워터마킹(P1).</t>
         </is>
       </c>
+      <c r="J348" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="25" t="n">
@@ -15750,6 +17537,11 @@
           <t>API Rate Limiting.</t>
         </is>
       </c>
+      <c r="J349" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="25" t="n">
@@ -15793,6 +17585,11 @@
           <t>Audit log 불변성(PostgreSQL append-only). 참고: docs/02 §2(access_logs), docs/03 §RLS</t>
         </is>
       </c>
+      <c r="J350" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="25" t="n">
@@ -15836,6 +17633,11 @@
           <t>키보드 네비게이션(WCAG 2.1 AA). 참고: docs/07 §9 접근성</t>
         </is>
       </c>
+      <c r="J351" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="25" t="n">
@@ -15879,6 +17681,11 @@
           <t>스크린 리더 호환(ARIA 레이블). 참고: docs/07 §9</t>
         </is>
       </c>
+      <c r="J352" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="25" t="n">
@@ -15922,6 +17729,11 @@
           <t>컬러 대비 4.5:1 검증. 참고: docs/07 §1 컬러 시스템·§9</t>
         </is>
       </c>
+      <c r="J353" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="25" t="n">
@@ -15965,6 +17777,11 @@
           <t>당사자 모드 TTS 통합. 참고: docs/07 §9 당사자 접근성 모드</t>
         </is>
       </c>
+      <c r="J354" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="24" t="n">
@@ -16008,6 +17825,11 @@
           <t>단위 테스트(Vitest, 핵심 로직 70%).</t>
         </is>
       </c>
+      <c r="J355" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="24" t="n">
@@ -16051,6 +17873,11 @@
           <t>API 통합 테스트(Supertest). 참고: docs/05 워크플로우</t>
         </is>
       </c>
+      <c r="J356" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="24" t="n">
@@ -16094,6 +17921,11 @@
           <t>E2E 테스트(Playwright, 5개 핵심 플로우). 참고: docs/06 §6 주요 플로우</t>
         </is>
       </c>
+      <c r="J357" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="24" t="n">
@@ -16137,6 +17969,11 @@
           <t>RLS 정책 자동 검증(pgTAP). 참고: docs/03 §RLS 정책 요약</t>
         </is>
       </c>
+      <c r="J358" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="24" t="n">
@@ -16180,6 +18017,11 @@
           <t>시각 회귀 테스트(Chromatic, P1). 참고: docs/07 디자인 시스템</t>
         </is>
       </c>
+      <c r="J359" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="24" t="n">
@@ -16223,6 +18065,11 @@
           <t>보호자 시나리오 — 가입~당사자 등록~권한 부여. 참고: docs/04 §1 보호자, bkit:zero-script-qa 스킬</t>
         </is>
       </c>
+      <c r="J360" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="24" t="n">
@@ -16266,6 +18113,11 @@
           <t>당사자 시나리오 — 자기표현 5일 연속. 참고: docs/04 §2 당사자</t>
         </is>
       </c>
+      <c r="J361" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="24" t="n">
@@ -16309,6 +18161,11 @@
           <t>활동지원사 시나리오 — 일지+인계 확인. 참고: docs/04 §3</t>
         </is>
       </c>
+      <c r="J362" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="24" t="n">
@@ -16352,6 +18209,11 @@
           <t>특수교사 시나리오 — IEP 작성+점검. 참고: docs/04 §4</t>
         </is>
       </c>
+      <c r="J363" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" s="24" t="n">
@@ -16395,6 +18257,11 @@
           <t>사회복지사 시나리오 — ISP·전환계획. 참고: docs/04 §5</t>
         </is>
       </c>
+      <c r="J364" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" s="24" t="n">
@@ -16438,6 +18305,11 @@
           <t>치료사 시나리오 — 계획서+회기+평가 사이클. 참고: docs/04 §6</t>
         </is>
       </c>
+      <c r="J365" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="24" t="n">
@@ -16481,6 +18353,11 @@
           <t>권한 외 접근 차단 검증. 참고: docs/05 §11 보안 흐름</t>
         </is>
       </c>
+      <c r="J366" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="24" t="n">
@@ -16524,6 +18401,11 @@
           <t>인수인계 권한 이양 검증. 참고: docs/05 §7</t>
         </is>
       </c>
+      <c r="J367" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="24" t="n">
@@ -16567,6 +18449,11 @@
           <t>타임라인 응답 성능(10k 기록, p95&lt;500ms). 참고: docs/02 §5 인덱스 전략</t>
         </is>
       </c>
+      <c r="J368" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="24" t="n">
@@ -16610,6 +18497,11 @@
           <t>권한 매트릭스 응답(20명, p95&lt;300ms).</t>
         </is>
       </c>
+      <c r="J369" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="24" t="n">
@@ -16653,6 +18545,11 @@
           <t>모바일 첫 화면 로드(LCP&lt;2.5s).</t>
         </is>
       </c>
+      <c r="J370" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="24" t="n">
@@ -16696,6 +18593,11 @@
           <t>부하 테스트(100 동시 일지 작성, P1).</t>
         </is>
       </c>
+      <c r="J371" s="43" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="13" t="n">
@@ -16739,6 +18641,11 @@
           <t>GitHub Actions — Lint·Type·Test 파이프라인. 참고: bkit:phase-9-deployment 스킬</t>
         </is>
       </c>
+      <c r="J372" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="13" t="n">
@@ -16782,6 +18689,11 @@
           <t>PR 미리보기 환경(Vercel Preview).</t>
         </is>
       </c>
+      <c r="J373" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="13" t="n">
@@ -16825,6 +18737,11 @@
           <t>DB 마이그레이션 검증(스테이징).</t>
         </is>
       </c>
+      <c r="J374" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="13" t="n">
@@ -16868,6 +18785,11 @@
           <t>모바일 EAS Build(iOS·Android).</t>
         </is>
       </c>
+      <c r="J375" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="13" t="n">
@@ -16911,6 +18833,11 @@
           <t>dev 환경 자동 배포.</t>
         </is>
       </c>
+      <c r="J376" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="13" t="n">
@@ -16954,6 +18881,11 @@
           <t>staging 환경 수동 배포 트리거.</t>
         </is>
       </c>
+      <c r="J377" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="13" t="n">
@@ -16997,6 +18929,11 @@
           <t>production 배포(승인 게이트).</t>
         </is>
       </c>
+      <c r="J378" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="13" t="n">
@@ -17040,6 +18977,11 @@
           <t>DB 백업 자동화(일 1회).</t>
         </is>
       </c>
+      <c r="J379" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="13" t="n">
@@ -17083,6 +19025,11 @@
           <t>롤백 시나리오 문서. 참고: bkit:rollback 스킬</t>
         </is>
       </c>
+      <c r="J380" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="13" t="n">
@@ -17126,6 +19073,11 @@
           <t>모니터링 대시보드(Grafana, P1).</t>
         </is>
       </c>
+      <c r="J381" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="13" t="n">
@@ -17169,6 +19121,11 @@
           <t>알림 인프라(PagerDuty/Slack, P1).</t>
         </is>
       </c>
+      <c r="J382" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="13" t="n">
@@ -17212,6 +19169,11 @@
           <t>로그 통합(Loki/Datadog, P1).</t>
         </is>
       </c>
+      <c r="J383" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="13" t="n">
@@ -17255,6 +19217,11 @@
           <t>분기별 외부 보안 감사(P1).</t>
         </is>
       </c>
+      <c r="J384" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="13" t="n">
@@ -17296,6 +19263,11 @@
       <c r="I385" s="33" t="inlineStr">
         <is>
           <t>GDPR/개인정보보호법 응대 워크플로우(데이터 열람·삭제 요청).</t>
+        </is>
+      </c>
+      <c r="J385" s="37" t="inlineStr">
+        <is>
+          <t>PL</t>
         </is>
       </c>
     </row>
@@ -17319,12 +19291,13 @@
       <c r="G386" s="26" t="n"/>
       <c r="H386" s="26" t="n"/>
       <c r="I386" s="34" t="n"/>
+      <c r="J386" s="34" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I385"/>
+  <autoFilter ref="A4:J385"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>